<commit_message>
Boost design & spreadsheet
</commit_message>
<xml_diff>
--- a/boost converter spread sheet.xlsx
+++ b/boost converter spread sheet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chihe\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\leonf\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{683BE410-0A57-4435-8C0A-8CE08AD16F9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17E56C08-6E6B-45E5-86EA-FEFAB76D08A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2985" yWindow="2985" windowWidth="21600" windowHeight="11460" activeTab="1" xr2:uid="{0EA872C3-4804-43CB-9F0B-5F94DB7B4351}"/>
+    <workbookView xWindow="780" yWindow="2055" windowWidth="21600" windowHeight="11295" xr2:uid="{0EA872C3-4804-43CB-9F0B-5F94DB7B4351}"/>
   </bookViews>
   <sheets>
     <sheet name="SS_Analysis" sheetId="1" r:id="rId1"/>
@@ -36,8 +36,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata">
+  <metadataTypes count="1">
+    <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLRICHVALUE" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <valueMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </valueMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="384" uniqueCount="157">
   <si>
     <t>Parameter</t>
   </si>
@@ -498,8 +520,17 @@
     <t>Rdc</t>
   </si>
   <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
     <t>4*piE-7</t>
-    <phoneticPr fontId="7" type="noConversion"/>
+    <phoneticPr fontId="0" type="noConversion"/>
+  </si>
+  <si>
+    <t>9</t>
   </si>
 </sst>
 </file>
@@ -507,23 +538,23 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="4">
-    <numFmt numFmtId="176" formatCode="0.0"/>
-    <numFmt numFmtId="177" formatCode="0.000E+00"/>
-    <numFmt numFmtId="178" formatCode="0.000"/>
-    <numFmt numFmtId="179" formatCode="0.00000"/>
+    <numFmt numFmtId="164" formatCode="0.0"/>
+    <numFmt numFmtId="165" formatCode="0.000E+00"/>
+    <numFmt numFmtId="166" formatCode="0.000"/>
+    <numFmt numFmtId="167" formatCode="0.00000"/>
   </numFmts>
   <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -531,7 +562,7 @@
       <b/>
       <sz val="11"/>
       <color theme="0"/>
-      <name val="等线"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -540,7 +571,7 @@
       <u/>
       <sz val="16"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -549,7 +580,7 @@
       <u/>
       <sz val="14"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -557,22 +588,21 @@
       <b/>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="12"/>
-      <name val="等线"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="9"/>
-      <name val="等线"/>
+      <sz val="11"/>
+      <color rgb="FF0F1115"/>
+      <name val="Consolas"/>
       <family val="3"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="6">
@@ -606,7 +636,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="57">
+  <borders count="59">
     <border>
       <left/>
       <right/>
@@ -975,8 +1005,8 @@
       <left style="thin">
         <color auto="1"/>
       </left>
-      <right style="thin">
-        <color auto="1"/>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
       </right>
       <top style="double">
         <color rgb="FF3F3F3F"/>
@@ -987,38 +1017,8 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="double">
         <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
       </left>
       <right style="thin">
         <color auto="1"/>
@@ -1337,6 +1337,54 @@
       <right style="thin">
         <color rgb="FF3F3F3F"/>
       </right>
+      <top/>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top/>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top/>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right/>
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
@@ -1346,49 +1394,32 @@
       <diagonal/>
     </border>
     <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
+      <left/>
+      <right style="double">
         <color rgb="FF3F3F3F"/>
       </right>
       <top/>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top/>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
       <right style="double">
         <color rgb="FF3F3F3F"/>
       </right>
-      <top/>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="double">
         <color rgb="FF3F3F3F"/>
       </right>
       <top/>
@@ -1398,15 +1429,30 @@
       <diagonal/>
     </border>
     <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top/>
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
       <bottom style="double">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1416,7 +1462,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="94">
+  <cellXfs count="98">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1454,7 +1500,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -1468,59 +1514,63 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="23" xfId="2" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="25" xfId="2" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="28" xfId="2" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="31" xfId="2" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="27" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="29" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="2" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="5" borderId="15" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="35" xfId="2" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="38" xfId="2" applyBorder="1"/>
-    <xf numFmtId="176" fontId="0" fillId="4" borderId="39" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="33" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="36" xfId="2" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="37" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="41" xfId="2" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="34" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="39" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="42" xfId="0" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="41" xfId="2" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="42" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="43" xfId="2" applyBorder="1"/>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="44" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="45" xfId="2" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="4" borderId="46" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="4" borderId="44" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="37" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="38" xfId="0" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="46" xfId="2" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="39" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="48" xfId="2" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="49" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="50" xfId="0" applyBorder="1"/>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="49" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="49" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="48" xfId="0" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="47" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="47" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="49" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="48" xfId="2" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="51" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="47" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="46" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="49" xfId="2" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="50" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="51" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="52" xfId="2" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="52" xfId="2" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="53" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="53" xfId="2" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="54" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="2" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="55" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="56" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="57" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="20% - Accent1" xfId="2" builtinId="30"/>
@@ -1538,6 +1588,125 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>95250</xdr:colOff>
+      <xdr:row>59</xdr:row>
+      <xdr:rowOff>66675</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>771525</xdr:colOff>
+      <xdr:row>93</xdr:row>
+      <xdr:rowOff>141957</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{928C74AF-CDCB-DA83-4B01-561098B30C55}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10029825" y="11896725"/>
+          <a:ext cx="7077075" cy="6676107"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
+<rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
+  <global>
+    <keyFlags>
+      <key name="_Self">
+        <flag name="ExcludeFromFile" value="1"/>
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_DisplayString">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Flags">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Format">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_SubLabel">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Attribution">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Icon">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Display">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_CanonicalPropertyNames">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_ClassificationId">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+    </keyFlags>
+  </global>
+</rvTypesInfo>
+</file>
+
+<file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
+  <rv s="0">
+    <v>0</v>
+    <v>5</v>
+  </rv>
+</rvData>
+</file>
+
+<file path=xl/richData/rdrichvaluestructure.xml><?xml version="1.0" encoding="utf-8"?>
+<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
+  <s t="_localImage">
+    <k n="_rvRel:LocalImageIdentifier" t="i"/>
+    <k n="CalcOrigin" t="i"/>
+  </s>
+</rvStructures>
+</file>
+
+<file path=xl/richData/richValueRel.xml><?xml version="1.0" encoding="utf-8"?>
+<richValueRels xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/richvaluerel" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <rel r:id="rId1"/>
+</richValueRels>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1857,25 +2026,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4C28CAE-7D6E-414C-9BF7-B54583CFEE9E}">
-  <dimension ref="A1:K103"/>
-  <sheetFormatPr defaultColWidth="12" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:O103"/>
+  <sheetFormatPr defaultColWidth="12" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.5" customWidth="1"/>
-    <col min="2" max="11" width="12.875" customWidth="1"/>
+    <col min="1" max="1" width="20.42578125" customWidth="1"/>
+    <col min="2" max="11" width="12.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="20.25" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="5" spans="1:3" ht="15.75" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="5" spans="1:3" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>0</v>
       </c>
@@ -1886,7 +2055,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A6" s="38" t="s">
         <v>37</v>
       </c>
@@ -1897,7 +2066,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="39" t="s">
         <v>38</v>
       </c>
@@ -1908,7 +2077,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="39" t="s">
         <v>39</v>
       </c>
@@ -1919,7 +2088,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="39" t="s">
         <v>57</v>
       </c>
@@ -1930,7 +2099,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="39" t="s">
         <v>58</v>
       </c>
@@ -1941,7 +2110,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="10" t="s">
         <v>5</v>
       </c>
@@ -1955,13 +2124,13 @@
     <row r="12" spans="1:3" ht="16.5" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A12" s="13"/>
     </row>
-    <row r="14" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="16" spans="1:3" ht="15.75" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="16" spans="1:3" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
         <v>0</v>
       </c>
@@ -1972,77 +2141,91 @@
         <v>7</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A17" s="46" t="s">
         <v>42</v>
       </c>
-      <c r="B17" s="47"/>
-      <c r="C17" s="48" t="s">
+      <c r="B17">
+        <v>0.5</v>
+      </c>
+      <c r="C17" s="47" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A18" s="49" t="s">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" s="48" t="s">
         <v>41</v>
       </c>
-      <c r="B18" s="50"/>
-      <c r="C18" s="51" t="s">
+      <c r="B18">
+        <v>0.33</v>
+      </c>
+      <c r="C18" s="49" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A19" s="59" t="s">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" s="57" t="s">
         <v>60</v>
       </c>
-      <c r="B19" s="60"/>
-      <c r="C19" s="61" t="s">
+      <c r="B19" s="58">
+        <v>1</v>
+      </c>
+      <c r="C19" s="59" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A20" s="52" t="s">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" s="50" t="s">
         <v>61</v>
       </c>
-      <c r="B20" s="53"/>
-      <c r="C20" s="54" t="s">
+      <c r="B20" s="51">
+        <v>0.1</v>
+      </c>
+      <c r="C20" s="52" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A21" s="55" t="s">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" s="53" t="s">
         <v>44</v>
       </c>
-      <c r="B21" s="16"/>
+      <c r="B21" s="16">
+        <v>0.33</v>
+      </c>
       <c r="C21" s="17" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A22" s="55" t="s">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" s="53" t="s">
         <v>45</v>
       </c>
-      <c r="B22" s="16"/>
+      <c r="B22" s="16">
+        <v>37</v>
+      </c>
       <c r="C22" s="18" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="90" t="s">
+    <row r="23" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="87" t="s">
         <v>104</v>
       </c>
-      <c r="B23" s="11"/>
+      <c r="B23" s="11">
+        <v>39</v>
+      </c>
       <c r="C23" s="19" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.2"/>
-    <row r="26" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="26" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="28" spans="1:3" ht="15.75" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="28" spans="1:3" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="3" t="s">
         <v>0</v>
       </c>
@@ -2053,7 +2236,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
         <v>10</v>
       </c>
@@ -2064,32 +2247,36 @@
         <v>3</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="B30" s="16"/>
+      <c r="B30" s="16">
+        <v>30</v>
+      </c>
       <c r="C30" s="17" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="B31" s="20"/>
+      <c r="B31" s="20">
+        <v>33</v>
+      </c>
       <c r="C31" s="19" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="32" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.2"/>
-    <row r="34" spans="1:11" ht="18" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="34" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="35" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="36" spans="1:11" ht="15.75" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="36" spans="1:15" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="3" t="s">
         <v>0</v>
       </c>
@@ -2124,7 +2311,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="37" spans="1:11" ht="15" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:15" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A37" s="4" t="s">
         <v>14</v>
       </c>
@@ -2140,7 +2327,7 @@
       <c r="E37" s="21" t="s">
         <v>3</v>
       </c>
-      <c r="F37" s="56">
+      <c r="F37" s="54">
         <v>5</v>
       </c>
       <c r="G37" s="21" t="s">
@@ -2159,7 +2346,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A38" s="45" t="s">
         <v>40</v>
       </c>
@@ -2175,7 +2362,7 @@
       <c r="E38" s="43" t="s">
         <v>3</v>
       </c>
-      <c r="F38" s="57">
+      <c r="F38" s="55">
         <v>3.5</v>
       </c>
       <c r="G38" s="43" t="s">
@@ -2194,7 +2381,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A39" s="7" t="s">
         <v>15</v>
       </c>
@@ -2212,7 +2399,7 @@
       <c r="E39" s="23" t="s">
         <v>4</v>
       </c>
-      <c r="F39" s="58">
+      <c r="F39" s="56">
         <v>0.5</v>
       </c>
       <c r="G39" s="23" t="s">
@@ -2231,107 +2418,170 @@
         <v>4</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A40" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="B40" s="25"/>
+      <c r="B40" s="25">
+        <f>B37^2/B39</f>
+        <v>50</v>
+      </c>
       <c r="C40" s="23" t="s">
         <v>113</v>
       </c>
-      <c r="D40" s="25"/>
+      <c r="D40" s="25">
+        <f t="shared" ref="D40:J40" si="0">D37^2/D39</f>
+        <v>50</v>
+      </c>
       <c r="E40" s="23" t="s">
         <v>113</v>
       </c>
-      <c r="F40" s="25"/>
+      <c r="F40" s="25">
+        <f t="shared" si="0"/>
+        <v>50</v>
+      </c>
       <c r="G40" s="23" t="s">
         <v>113</v>
       </c>
-      <c r="H40" s="25"/>
+      <c r="H40" s="25">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
       <c r="I40" s="23" t="s">
         <v>113</v>
       </c>
-      <c r="J40" s="25"/>
+      <c r="J40" s="25">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
       <c r="K40" s="23" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A41" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="B41" s="25"/>
+      <c r="B41" s="25">
+        <f>1-B38/B37</f>
+        <v>0.5</v>
+      </c>
       <c r="C41" s="23" t="s">
         <v>114</v>
       </c>
-      <c r="D41" s="25"/>
+      <c r="D41" s="25">
+        <f t="shared" ref="D41:J41" si="1">1-D38/D37</f>
+        <v>0.33399999999999996</v>
+      </c>
       <c r="E41" s="23" t="s">
         <v>114</v>
       </c>
-      <c r="F41" s="25"/>
+      <c r="F41" s="25">
+        <f t="shared" si="1"/>
+        <v>0.30000000000000004</v>
+      </c>
       <c r="G41" s="23" t="s">
         <v>114</v>
       </c>
-      <c r="H41" s="25"/>
+      <c r="H41" s="25">
+        <f t="shared" si="1"/>
+        <v>0.5</v>
+      </c>
       <c r="I41" s="23" t="s">
         <v>114</v>
       </c>
-      <c r="J41" s="25"/>
+      <c r="J41" s="25">
+        <f t="shared" si="1"/>
+        <v>0.30000000000000004</v>
+      </c>
       <c r="K41" s="23" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A42" s="39" t="s">
         <v>47</v>
       </c>
-      <c r="B42" s="25"/>
+      <c r="B42" s="25">
+        <f>B47/(1-B41)</f>
+        <v>0.2</v>
+      </c>
       <c r="C42" s="23" t="s">
         <v>115</v>
       </c>
-      <c r="D42" s="25"/>
+      <c r="D42" s="25">
+        <f t="shared" ref="D42:J42" si="2">D47/(1-D41)</f>
+        <v>0.15015015015015015</v>
+      </c>
       <c r="E42" s="23" t="s">
         <v>115</v>
       </c>
-      <c r="F42" s="25"/>
+      <c r="F42" s="25">
+        <f t="shared" si="2"/>
+        <v>0.14285714285714288</v>
+      </c>
       <c r="G42" s="23" t="s">
         <v>115</v>
       </c>
-      <c r="H42" s="25"/>
+      <c r="H42" s="25">
+        <f t="shared" si="2"/>
+        <v>2</v>
+      </c>
       <c r="I42" s="23" t="s">
         <v>115</v>
       </c>
-      <c r="J42" s="25"/>
+      <c r="J42" s="25">
+        <f t="shared" si="2"/>
+        <v>1.4285714285714286</v>
+      </c>
       <c r="K42" s="23" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="O42">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A43" s="39" t="s">
         <v>46</v>
       </c>
-      <c r="B43" s="25"/>
+      <c r="B43" s="25">
+        <f>(B37-B38)*(1-B41)/($B$23/1000000*($B$11*1000))</f>
+        <v>0.32051282051282054</v>
+      </c>
       <c r="C43" s="23" t="s">
         <v>116</v>
       </c>
-      <c r="D43" s="25"/>
+      <c r="D43" s="25">
+        <f t="shared" ref="D43:J43" si="3">(D37-D38)*(1-D41)/($B$23/1000000*($B$11*1000))</f>
+        <v>0.28518461538461537</v>
+      </c>
       <c r="E43" s="23" t="s">
         <v>116</v>
       </c>
-      <c r="F43" s="25"/>
+      <c r="F43" s="25">
+        <f t="shared" si="3"/>
+        <v>0.26923076923076922</v>
+      </c>
       <c r="G43" s="23" t="s">
         <v>116</v>
       </c>
-      <c r="H43" s="25"/>
+      <c r="H43" s="25">
+        <f t="shared" si="3"/>
+        <v>0.32051282051282054</v>
+      </c>
       <c r="I43" s="23" t="s">
         <v>116</v>
       </c>
-      <c r="J43" s="25"/>
+      <c r="J43" s="25">
+        <f t="shared" si="3"/>
+        <v>0.26923076923076922</v>
+      </c>
       <c r="K43" s="23" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A44" s="7" t="s">
         <v>18</v>
       </c>
@@ -2341,241 +2591,361 @@
       </c>
       <c r="C44" s="23"/>
       <c r="D44" s="26" t="str">
-        <f>IF(D42&gt;=D43/2,"Yes","No")</f>
+        <f t="shared" ref="D44:J44" si="4">IF(D42&gt;=D43/2,"Yes","No")</f>
         <v>Yes</v>
       </c>
       <c r="E44" s="23"/>
       <c r="F44" s="26" t="str">
-        <f>IF(F42&gt;=F43/2,"Yes","No")</f>
+        <f t="shared" si="4"/>
         <v>Yes</v>
       </c>
       <c r="G44" s="23"/>
       <c r="H44" s="26" t="str">
-        <f>IF(H42&gt;=H43/2,"Yes","No")</f>
+        <f t="shared" si="4"/>
         <v>Yes</v>
       </c>
       <c r="I44" s="23"/>
       <c r="J44" s="26" t="str">
-        <f>IF(J42&gt;=J43/2,"Yes","No")</f>
+        <f t="shared" si="4"/>
         <v>Yes</v>
       </c>
       <c r="K44" s="24"/>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A45" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="B45" s="25"/>
+      <c r="B45" s="25">
+        <f>B42+B38*B41/(2*$B$23/1000000*$B$11*1000)</f>
+        <v>0.36025641025641031</v>
+      </c>
       <c r="C45" s="23" t="s">
         <v>117</v>
       </c>
-      <c r="D45" s="25"/>
+      <c r="D45" s="25">
+        <f t="shared" ref="D45:J45" si="5">D42+D38*D41/(2*$B$23/1000000*$B$11*1000)</f>
+        <v>0.29274245784245784</v>
+      </c>
       <c r="E45" s="23" t="s">
         <v>117</v>
       </c>
-      <c r="F45" s="25"/>
+      <c r="F45" s="25">
+        <f t="shared" si="5"/>
+        <v>0.27747252747252754</v>
+      </c>
       <c r="G45" s="23" t="s">
         <v>117</v>
       </c>
-      <c r="H45" s="25"/>
+      <c r="H45" s="25">
+        <f t="shared" si="5"/>
+        <v>2.1602564102564101</v>
+      </c>
       <c r="I45" s="23" t="s">
         <v>117</v>
       </c>
-      <c r="J45" s="25"/>
+      <c r="J45" s="25">
+        <f t="shared" si="5"/>
+        <v>1.5631868131868132</v>
+      </c>
       <c r="K45" s="23" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A46" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="B46" s="25"/>
+      <c r="B46">
+        <f>SQRT(B42^2 + (B43^2)/12)</f>
+        <v>0.22036493749253827</v>
+      </c>
       <c r="C46" s="23" t="s">
         <v>118</v>
       </c>
-      <c r="D46" s="25"/>
+      <c r="D46">
+        <f t="shared" ref="D46:J46" si="6">SQRT(D42^2 + (D43^2)/12)</f>
+        <v>0.17123840007754848</v>
+      </c>
       <c r="E46" s="23" t="s">
         <v>118</v>
       </c>
-      <c r="F46" s="25"/>
+      <c r="F46">
+        <f t="shared" si="6"/>
+        <v>0.16263024684958036</v>
+      </c>
       <c r="G46" s="23" t="s">
         <v>118</v>
       </c>
-      <c r="H46" s="25"/>
+      <c r="H46">
+        <f t="shared" si="6"/>
+        <v>2.0021390325539556</v>
+      </c>
       <c r="I46" s="23" t="s">
         <v>118</v>
       </c>
-      <c r="J46" s="25"/>
+      <c r="J46">
+        <f t="shared" si="6"/>
+        <v>1.430684018382697</v>
+      </c>
       <c r="K46" s="23" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A47" s="28" t="s">
         <v>50</v>
       </c>
-      <c r="B47" s="29"/>
+      <c r="B47" s="29">
+        <f>B39/B37</f>
+        <v>0.1</v>
+      </c>
       <c r="C47" s="23" t="s">
         <v>119</v>
       </c>
-      <c r="D47" s="29"/>
+      <c r="D47" s="29">
+        <f t="shared" ref="D47:J47" si="7">D39/D37</f>
+        <v>0.1</v>
+      </c>
       <c r="E47" s="23" t="s">
         <v>119</v>
       </c>
-      <c r="F47" s="29"/>
+      <c r="F47" s="29">
+        <f t="shared" si="7"/>
+        <v>0.1</v>
+      </c>
       <c r="G47" s="23" t="s">
         <v>119</v>
       </c>
-      <c r="H47" s="29"/>
+      <c r="H47" s="29">
+        <f t="shared" si="7"/>
+        <v>1</v>
+      </c>
       <c r="I47" s="23" t="s">
         <v>119</v>
       </c>
-      <c r="J47" s="29"/>
+      <c r="J47" s="29">
+        <f t="shared" si="7"/>
+        <v>1</v>
+      </c>
       <c r="K47" s="23" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A48" s="28" t="s">
         <v>52</v>
       </c>
-      <c r="B48" s="29"/>
+      <c r="B48" s="29">
+        <f>SQRT(B41)*B46</f>
+        <v>0.15582154163672349</v>
+      </c>
       <c r="C48" s="23" t="s">
         <v>120</v>
       </c>
-      <c r="D48" s="29"/>
+      <c r="D48" s="29">
+        <f t="shared" ref="D48:J48" si="8">SQRT(D41)*D46</f>
+        <v>9.8963351533856186E-2</v>
+      </c>
       <c r="E48" s="23" t="s">
         <v>120</v>
       </c>
-      <c r="F48" s="29"/>
+      <c r="F48" s="29">
+        <f t="shared" si="8"/>
+        <v>8.9076254732148655E-2</v>
+      </c>
       <c r="G48" s="23" t="s">
         <v>120</v>
       </c>
-      <c r="H48" s="29"/>
+      <c r="H48" s="29">
+        <f t="shared" si="8"/>
+        <v>1.4157260867971759</v>
+      </c>
       <c r="I48" s="23" t="s">
         <v>120</v>
       </c>
-      <c r="J48" s="29"/>
+      <c r="J48" s="29">
+        <f t="shared" si="8"/>
+        <v>0.78361790953033894</v>
+      </c>
       <c r="K48" s="23" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" s="28" t="s">
         <v>51</v>
       </c>
-      <c r="B49" s="29"/>
+      <c r="B49" s="29">
+        <f>SQRT((1 - B41) * B46^2 - B47^2)</f>
+        <v>0.11950043028393306</v>
+      </c>
       <c r="C49" s="23" t="s">
         <v>121</v>
       </c>
-      <c r="D49" s="29"/>
+      <c r="D49" s="29">
+        <f t="shared" ref="D49:J49" si="9">SQRT((1 - D41) * D46^2 - D47^2)</f>
+        <v>9.7615801560530957E-2</v>
+      </c>
       <c r="E49" s="23" t="s">
         <v>121</v>
       </c>
-      <c r="F49" s="29"/>
+      <c r="F49" s="29">
+        <f t="shared" si="9"/>
+        <v>9.2271436713908403E-2</v>
+      </c>
       <c r="G49" s="23" t="s">
         <v>121</v>
       </c>
-      <c r="H49" s="29"/>
+      <c r="H49" s="29">
+        <f t="shared" si="9"/>
+        <v>1.0021378911297809</v>
+      </c>
       <c r="I49" s="23" t="s">
         <v>121</v>
       </c>
-      <c r="J49" s="29"/>
+      <c r="J49" s="29">
+        <f t="shared" si="9"/>
+        <v>0.65787516469233187</v>
+      </c>
       <c r="K49" s="23" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="B50" s="29"/>
+      <c r="B50" s="29">
+        <f>B37</f>
+        <v>5</v>
+      </c>
       <c r="C50" s="23" t="s">
         <v>122</v>
       </c>
-      <c r="D50" s="29"/>
+      <c r="D50" s="29">
+        <f t="shared" ref="D50:J50" si="10">D37</f>
+        <v>5</v>
+      </c>
       <c r="E50" s="23" t="s">
         <v>122</v>
       </c>
-      <c r="F50" s="29"/>
+      <c r="F50" s="29">
+        <f t="shared" si="10"/>
+        <v>5</v>
+      </c>
       <c r="G50" s="23" t="s">
         <v>122</v>
       </c>
-      <c r="H50" s="29"/>
+      <c r="H50" s="29">
+        <f t="shared" si="10"/>
+        <v>5</v>
+      </c>
       <c r="I50" s="23" t="s">
         <v>122</v>
       </c>
-      <c r="J50" s="29"/>
+      <c r="J50" s="29">
+        <f t="shared" si="10"/>
+        <v>5</v>
+      </c>
       <c r="K50" s="23" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" s="28" t="s">
         <v>54</v>
       </c>
-      <c r="B51" s="29"/>
+      <c r="B51" s="29">
+        <f>B37</f>
+        <v>5</v>
+      </c>
       <c r="C51" s="23" t="s">
         <v>123</v>
       </c>
-      <c r="D51" s="29"/>
+      <c r="D51" s="29">
+        <f t="shared" ref="D51:J51" si="11">D37</f>
+        <v>5</v>
+      </c>
       <c r="E51" s="23" t="s">
         <v>123</v>
       </c>
-      <c r="F51" s="29"/>
+      <c r="F51" s="29">
+        <f t="shared" si="11"/>
+        <v>5</v>
+      </c>
       <c r="G51" s="23" t="s">
         <v>123</v>
       </c>
-      <c r="H51" s="29"/>
+      <c r="H51" s="29">
+        <f t="shared" si="11"/>
+        <v>5</v>
+      </c>
       <c r="I51" s="23" t="s">
         <v>123</v>
       </c>
-      <c r="J51" s="29"/>
+      <c r="J51" s="29">
+        <f t="shared" si="11"/>
+        <v>5</v>
+      </c>
       <c r="K51" s="23" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="52" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A52" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="B52" s="20"/>
+      <c r="B52" s="20">
+        <f xml:space="preserve"> (B47 * B41) / ($B$31 /1000000* $B$11 * 1000)*1000</f>
+        <v>15.151515151515152</v>
+      </c>
       <c r="C52" s="31" t="s">
         <v>124</v>
       </c>
-      <c r="D52" s="20"/>
+      <c r="D52" s="20">
+        <f xml:space="preserve"> (D47 * D41) / ($B$31 /1000000* $B$11 * 1000)*1000</f>
+        <v>10.121212121212119</v>
+      </c>
       <c r="E52" s="31" t="s">
         <v>124</v>
       </c>
-      <c r="F52" s="20"/>
+      <c r="F52" s="20">
+        <f xml:space="preserve"> (F47 * F41) / ($B$31 /1000000* $B$11 * 1000)*1000</f>
+        <v>9.0909090909090917</v>
+      </c>
       <c r="G52" s="31" t="s">
         <v>124</v>
       </c>
-      <c r="H52" s="20"/>
+      <c r="H52" s="20">
+        <f xml:space="preserve"> (H47 * H41) / ($B$31 /1000000* $B$11 * 1000)*1000</f>
+        <v>151.5151515151515</v>
+      </c>
       <c r="I52" s="31" t="s">
         <v>124</v>
       </c>
-      <c r="J52" s="20"/>
+      <c r="J52" s="20">
+        <f xml:space="preserve"> (J47 * J41) / ($B$31 /1000000* $B$11 * 1000)*1000</f>
+        <v>90.909090909090907</v>
+      </c>
       <c r="K52" s="31" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="53" spans="1:11" ht="15" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="B53" s="33"/>
       <c r="C53" s="34"/>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B54" s="33"/>
       <c r="C54" s="34"/>
     </row>
-    <row r="55" spans="1:11" ht="18" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="56" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="57" spans="1:11" ht="15.75" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="57" spans="1:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A57" s="3" t="s">
         <v>0</v>
       </c>
@@ -2606,370 +2976,492 @@
         <v>7</v>
       </c>
     </row>
-    <row r="58" spans="1:11" ht="15" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A58" s="7" t="s">
         <v>16</v>
       </c>
       <c r="B58" s="8">
         <f>B40</f>
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="C58" s="23" t="s">
         <v>20</v>
       </c>
       <c r="D58" s="8">
         <f>D40</f>
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="E58" s="23" t="s">
         <v>20</v>
       </c>
       <c r="F58" s="8">
         <f>F40</f>
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="G58" s="23" t="s">
         <v>20</v>
       </c>
       <c r="H58" s="8">
         <f>H40</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I58" s="23" t="s">
         <v>20</v>
       </c>
       <c r="J58" s="8">
         <f>J40</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="K58" s="24" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" s="7" t="s">
         <v>17</v>
       </c>
       <c r="B59" s="8">
         <f>B41</f>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="C59" s="23"/>
       <c r="D59" s="8">
         <f>D41</f>
-        <v>0</v>
+        <v>0.33399999999999996</v>
       </c>
       <c r="E59" s="23"/>
       <c r="F59" s="8">
         <f>F41</f>
-        <v>0</v>
+        <v>0.30000000000000004</v>
       </c>
       <c r="G59" s="23"/>
       <c r="H59" s="8">
         <f>H41</f>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="I59" s="23"/>
       <c r="J59" s="8">
         <f>J41</f>
-        <v>0</v>
+        <v>0.30000000000000004</v>
       </c>
       <c r="K59" s="24"/>
     </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="B60" s="25"/>
+      <c r="B60" s="25">
+        <v>5</v>
+      </c>
       <c r="C60" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="D60" s="25"/>
+      <c r="D60" s="25">
+        <v>5</v>
+      </c>
       <c r="E60" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="F60" s="23"/>
+      <c r="F60" s="88">
+        <v>5</v>
+      </c>
       <c r="G60" s="23"/>
-      <c r="H60" s="25"/>
+      <c r="H60" s="25">
+        <v>5</v>
+      </c>
       <c r="I60" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="J60" s="25"/>
+      <c r="J60" s="25">
+        <v>5</v>
+      </c>
       <c r="K60" s="24" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="B61" s="25"/>
-      <c r="C61" s="23" t="s">
+      <c r="B61" s="25">
+        <v>0.5</v>
+      </c>
+      <c r="C61" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="D61" s="25"/>
-      <c r="E61" s="23" t="s">
+      <c r="D61" s="25">
+        <v>0.33400000000000002</v>
+      </c>
+      <c r="E61" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="F61" s="23"/>
-      <c r="G61" s="23"/>
-      <c r="H61" s="25"/>
-      <c r="I61" s="23" t="s">
+      <c r="F61" s="25">
+        <v>0.3</v>
+      </c>
+      <c r="G61" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="J61" s="25"/>
+      <c r="H61" s="25">
+        <v>0.5</v>
+      </c>
+      <c r="I61" s="24" t="s">
+        <v>4</v>
+      </c>
+      <c r="J61" s="25">
+        <v>0.3</v>
+      </c>
       <c r="K61" s="24" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="B62" s="27"/>
+      <c r="B62" s="27" t="s">
+        <v>153</v>
+      </c>
       <c r="C62" s="23"/>
-      <c r="D62" s="27"/>
+      <c r="D62" s="27" t="s">
+        <v>153</v>
+      </c>
       <c r="E62" s="23"/>
-      <c r="F62" s="23"/>
+      <c r="F62" s="25" t="s">
+        <v>153</v>
+      </c>
       <c r="G62" s="23"/>
-      <c r="H62" s="27"/>
+      <c r="H62" s="27" t="s">
+        <v>153</v>
+      </c>
       <c r="I62" s="23"/>
-      <c r="J62" s="27"/>
+      <c r="J62" s="27" t="s">
+        <v>153</v>
+      </c>
       <c r="K62" s="24"/>
     </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" s="39" t="s">
         <v>46</v>
       </c>
-      <c r="B63" s="27"/>
+      <c r="B63" s="27">
+        <v>0.37</v>
+      </c>
       <c r="C63" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="D63" s="27"/>
+      <c r="D63" s="27">
+        <v>0.28000000000000003</v>
+      </c>
       <c r="E63" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="F63" s="23"/>
+      <c r="F63" s="88">
+        <v>0.26</v>
+      </c>
       <c r="G63" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="H63" s="27"/>
+      <c r="H63" s="27">
+        <v>0.32</v>
+      </c>
       <c r="I63" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="J63" s="27"/>
+      <c r="J63" s="27">
+        <v>0.24</v>
+      </c>
       <c r="K63" s="23" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="B64" s="25"/>
+      <c r="B64" s="25">
+        <v>0.37</v>
+      </c>
       <c r="C64" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="D64" s="25"/>
+      <c r="D64" s="27">
+        <v>0.28999999999999998</v>
+      </c>
       <c r="E64" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="F64" s="23"/>
+      <c r="F64" s="88">
+        <v>0.28000000000000003</v>
+      </c>
       <c r="G64" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="H64" s="25"/>
+      <c r="H64" s="25">
+        <v>2.17</v>
+      </c>
       <c r="I64" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="J64" s="25"/>
+      <c r="J64" s="25">
+        <v>1.59</v>
+      </c>
       <c r="K64" s="23" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="B65" s="25"/>
+      <c r="B65" s="25">
+        <v>0.23</v>
+      </c>
       <c r="C65" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="D65" s="25"/>
+      <c r="D65" s="25">
+        <v>0.17</v>
+      </c>
       <c r="E65" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="F65" s="23"/>
+      <c r="F65" s="88">
+        <v>0.16</v>
+      </c>
       <c r="G65" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="H65" s="25"/>
+      <c r="H65" s="25">
+        <v>2.0699999999999998</v>
+      </c>
       <c r="I65" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="J65" s="25"/>
+      <c r="J65" s="25">
+        <v>1.59</v>
+      </c>
       <c r="K65" s="23" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66" s="28" t="s">
         <v>50</v>
       </c>
-      <c r="B66" s="29"/>
+      <c r="B66" s="29">
+        <v>0.1</v>
+      </c>
       <c r="C66" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="D66" s="29"/>
+      <c r="D66" s="29">
+        <v>0.1</v>
+      </c>
       <c r="E66" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="F66" s="30"/>
+      <c r="F66" s="29">
+        <v>0.1</v>
+      </c>
       <c r="G66" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="H66" s="29"/>
+      <c r="H66" s="29">
+        <v>1</v>
+      </c>
       <c r="I66" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="J66" s="29"/>
+      <c r="J66" s="29">
+        <v>1</v>
+      </c>
       <c r="K66" s="23" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" s="28" t="s">
         <v>52</v>
       </c>
-      <c r="B67" s="29"/>
+      <c r="B67" s="29">
+        <v>0.17</v>
+      </c>
       <c r="C67" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="D67" s="29"/>
+      <c r="D67" s="29">
+        <v>0.1</v>
+      </c>
       <c r="E67" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="F67" s="30"/>
+      <c r="F67" s="29">
+        <v>0.1</v>
+      </c>
       <c r="G67" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="H67" s="29"/>
+      <c r="H67" s="29">
+        <v>1.6</v>
+      </c>
       <c r="I67" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="J67" s="29"/>
+      <c r="J67" s="29">
+        <v>0.97</v>
+      </c>
       <c r="K67" s="23" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" s="28" t="s">
         <v>51</v>
       </c>
-      <c r="B68" s="29"/>
+      <c r="B68" s="29">
+        <v>0.12</v>
+      </c>
       <c r="C68" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="D68" s="29"/>
+      <c r="D68" s="29">
+        <v>0.1</v>
+      </c>
       <c r="E68" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="F68" s="30"/>
+      <c r="F68" s="29">
+        <v>0.1</v>
+      </c>
       <c r="G68" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="H68" s="29"/>
+      <c r="H68" s="29">
+        <v>1</v>
+      </c>
       <c r="I68" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="J68" s="29"/>
+      <c r="J68" s="29">
+        <v>0.77</v>
+      </c>
       <c r="K68" s="23" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="B69" s="29"/>
+      <c r="B69" s="29">
+        <v>5.03</v>
+      </c>
       <c r="C69" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="D69" s="29"/>
+      <c r="D69" s="29">
+        <v>5.01</v>
+      </c>
       <c r="E69" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="F69" s="30"/>
+      <c r="F69" s="29">
+        <v>5.01</v>
+      </c>
       <c r="G69" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="H69" s="29"/>
+      <c r="H69" s="29">
+        <v>5.03</v>
+      </c>
       <c r="I69" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="J69" s="29"/>
+      <c r="J69" s="29">
+        <v>5.05</v>
+      </c>
       <c r="K69" s="23" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" s="28" t="s">
         <v>54</v>
       </c>
-      <c r="B70" s="29"/>
+      <c r="B70" s="29">
+        <v>5</v>
+      </c>
       <c r="C70" s="30" t="s">
         <v>3</v>
       </c>
-      <c r="D70" s="29"/>
+      <c r="D70" s="29">
+        <v>5</v>
+      </c>
       <c r="E70" s="30" t="s">
         <v>3</v>
       </c>
-      <c r="F70" s="30"/>
+      <c r="F70" s="29">
+        <v>5</v>
+      </c>
       <c r="G70" s="30" t="s">
         <v>3</v>
       </c>
-      <c r="H70" s="29"/>
+      <c r="H70" s="29">
+        <v>5.0199999999999996</v>
+      </c>
       <c r="I70" s="30" t="s">
         <v>3</v>
       </c>
-      <c r="J70" s="29"/>
+      <c r="J70" s="29">
+        <v>5</v>
+      </c>
       <c r="K70" s="30" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="71" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A71" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="B71" s="20"/>
+      <c r="B71" s="20">
+        <v>7.0000000000000007E-2</v>
+      </c>
       <c r="C71" s="31" t="s">
         <v>3</v>
       </c>
-      <c r="D71" s="20"/>
+      <c r="D71" s="20">
+        <v>0.04</v>
+      </c>
       <c r="E71" s="31" t="s">
         <v>3</v>
       </c>
-      <c r="F71" s="31"/>
+      <c r="F71" s="20">
+        <v>0.04</v>
+      </c>
       <c r="G71" s="31" t="s">
         <v>3</v>
       </c>
-      <c r="H71" s="20"/>
+      <c r="H71" s="20">
+        <v>0.08</v>
+      </c>
       <c r="I71" s="31" t="s">
         <v>3</v>
       </c>
-      <c r="J71" s="20"/>
+      <c r="J71" s="20">
+        <v>0.1</v>
+      </c>
       <c r="K71" s="31" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="72" spans="1:11" ht="15" thickTop="1" x14ac:dyDescent="0.2"/>
-    <row r="74" spans="1:11" ht="18" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="74" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A74" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="75" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="76" spans="1:11" ht="15.75" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="76" spans="1:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A76" s="3" t="s">
         <v>0</v>
       </c>
@@ -2980,7 +3472,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="77" spans="1:11" ht="15" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A77" s="4" t="s">
         <v>127</v>
       </c>
@@ -2991,7 +3483,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A78" s="15" t="s">
         <v>128</v>
       </c>
@@ -3002,7 +3494,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79" s="15" t="s">
         <v>23</v>
       </c>
@@ -3014,7 +3506,7 @@
       </c>
     </row>
     <row r="80" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A80" s="55" t="s">
+      <c r="A80" s="53" t="s">
         <v>133</v>
       </c>
       <c r="B80" s="37">
@@ -3024,8 +3516,8 @@
         <v>24</v>
       </c>
     </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A81" s="55" t="s">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A81" s="53" t="s">
         <v>132</v>
       </c>
       <c r="B81" s="35">
@@ -3035,79 +3527,95 @@
         <v>25</v>
       </c>
     </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A82" s="55" t="s">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A82" s="53" t="s">
         <v>131</v>
       </c>
-      <c r="B82" s="16"/>
+      <c r="B82" s="16">
+        <v>18</v>
+      </c>
       <c r="C82" s="18" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A83" s="55" t="s">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A83" s="53" t="s">
         <v>130</v>
       </c>
-      <c r="B83" s="16"/>
+      <c r="B83" s="16">
+        <v>0.47</v>
+      </c>
       <c r="C83" s="18" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A84" s="55" t="s">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A84" s="53" t="s">
         <v>134</v>
       </c>
-      <c r="B84" s="16"/>
+      <c r="B84" s="16">
+        <v>4.7</v>
+      </c>
       <c r="C84" s="18" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A85" s="55" t="s">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A85" s="53" t="s">
         <v>135</v>
       </c>
-      <c r="B85" s="16"/>
+      <c r="B85" s="16">
+        <v>270</v>
+      </c>
       <c r="C85" s="18" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A86" s="55" t="s">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A86" s="53" t="s">
         <v>136</v>
       </c>
-      <c r="B86" s="16"/>
+      <c r="B86" s="16">
+        <v>1000</v>
+      </c>
       <c r="C86" s="18" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A87" s="55" t="s">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A87" s="53" t="s">
         <v>27</v>
       </c>
-      <c r="B87" s="16"/>
+      <c r="B87" s="16">
+        <v>10</v>
+      </c>
       <c r="C87" s="18" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A88" s="55" t="s">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A88" s="53" t="s">
         <v>28</v>
       </c>
-      <c r="B88" s="16"/>
+      <c r="B88" s="16">
+        <v>10</v>
+      </c>
       <c r="C88" s="18" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A89" s="55" t="s">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A89" s="53" t="s">
         <v>129</v>
       </c>
-      <c r="B89" s="16"/>
+      <c r="B89" s="16">
+        <v>1000</v>
+      </c>
       <c r="C89" s="18" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90" s="15" t="s">
         <v>125</v>
       </c>
@@ -3118,7 +3626,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91" s="15" t="s">
         <v>126</v>
       </c>
@@ -3128,29 +3636,36 @@
       <c r="C91" s="18" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="E91" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A92" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="B92" s="16"/>
+      <c r="B92" s="16">
+        <v>0.15</v>
+      </c>
       <c r="C92" s="18"/>
     </row>
-    <row r="93" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A93" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="B93" s="20"/>
+      <c r="B93" s="20">
+        <v>190</v>
+      </c>
       <c r="C93" s="19"/>
     </row>
-    <row r="94" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.2"/>
-    <row r="96" spans="1:3" ht="18" x14ac:dyDescent="0.25">
-      <c r="A96" s="2" t="s">
+    <row r="94" spans="1:5" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="95" spans="1:5" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A95" s="2" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="97" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="98" spans="1:11" ht="15.75" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="98" spans="1:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A98" s="3" t="s">
         <v>0</v>
       </c>
@@ -3181,47 +3696,47 @@
         <v>7</v>
       </c>
     </row>
-    <row r="99" spans="1:11" ht="15" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A99" s="7" t="s">
         <v>16</v>
       </c>
       <c r="B99" s="8">
         <f>B40</f>
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="C99" s="23" t="s">
         <v>20</v>
       </c>
       <c r="D99" s="8">
         <f>D40</f>
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="E99" s="23" t="s">
         <v>20</v>
       </c>
       <c r="F99" s="8">
         <f>F40</f>
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="G99" s="23" t="s">
         <v>20</v>
       </c>
       <c r="H99" s="8">
         <f>H40</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I99" s="23" t="s">
         <v>20</v>
       </c>
       <c r="J99" s="8">
         <f>J40</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="K99" s="24" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="100" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A100" s="7" t="s">
         <v>33</v>
       </c>
@@ -3256,85 +3771,105 @@
         <v>3</v>
       </c>
     </row>
-    <row r="101" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A101" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="B101" s="25"/>
+      <c r="B101" s="25">
+        <v>5</v>
+      </c>
       <c r="C101" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="D101" s="25"/>
+      <c r="D101" s="25">
+        <v>5</v>
+      </c>
       <c r="E101" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="F101" s="23"/>
+      <c r="F101" s="23" t="s">
+        <v>154</v>
+      </c>
       <c r="G101" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="H101" s="25"/>
+      <c r="H101" s="25">
+        <v>5</v>
+      </c>
       <c r="I101" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="J101" s="25"/>
+      <c r="J101" s="25">
+        <v>5</v>
+      </c>
       <c r="K101" s="24" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="102" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A102" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="B102" s="20"/>
+      <c r="B102" s="20">
+        <v>5</v>
+      </c>
       <c r="C102" s="31" t="s">
         <v>36</v>
       </c>
-      <c r="D102" s="20"/>
+      <c r="D102" s="20">
+        <v>8</v>
+      </c>
       <c r="E102" s="31" t="s">
         <v>36</v>
       </c>
-      <c r="F102" s="31"/>
+      <c r="F102" s="31" t="s">
+        <v>156</v>
+      </c>
       <c r="G102" s="31" t="s">
         <v>36</v>
       </c>
-      <c r="H102" s="20"/>
+      <c r="H102" s="20">
+        <v>30</v>
+      </c>
       <c r="I102" s="31" t="s">
         <v>36</v>
       </c>
-      <c r="J102" s="20"/>
+      <c r="J102" s="20">
+        <v>15</v>
+      </c>
       <c r="K102" s="32" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="103" spans="1:11" ht="15" thickTop="1" x14ac:dyDescent="0.2"/>
+    <row r="103" spans="1:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F74A05D-7210-44AC-859D-2846F0884F7B}">
   <dimension ref="A1:G52"/>
-  <sheetFormatPr defaultColWidth="12" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="12" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.5" customWidth="1"/>
-    <col min="2" max="9" width="12.875" customWidth="1"/>
+    <col min="1" max="1" width="24.42578125" customWidth="1"/>
+    <col min="2" max="9" width="12.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="20.25" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="5" spans="1:3" ht="15.75" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="5" spans="1:3" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>0</v>
       </c>
@@ -3345,51 +3880,55 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A6" s="38" t="s">
         <v>104</v>
       </c>
       <c r="B6" s="5">
-        <v>0.39</v>
+        <f>SS_Analysis!B23</f>
+        <v>39</v>
       </c>
       <c r="C6" s="18" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="39" t="s">
         <v>94</v>
       </c>
       <c r="B7" s="8">
+        <f>SS_Analysis!H42</f>
         <v>2</v>
       </c>
       <c r="C7" s="9" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="39" t="s">
         <v>95</v>
       </c>
       <c r="B8" s="8">
-        <v>2.16</v>
+        <f>SS_Analysis!H45</f>
+        <v>2.1602564102564101</v>
       </c>
       <c r="C8" s="9" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="39" t="s">
         <v>93</v>
       </c>
       <c r="B9" s="8">
-        <v>2.0019999999999998</v>
+        <f>SS_Analysis!H46</f>
+        <v>2.0021390325539556</v>
       </c>
       <c r="C9" s="9" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
         <v>63</v>
       </c>
@@ -3400,7 +3939,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="10" t="s">
         <v>5</v>
       </c>
@@ -3415,15 +3954,15 @@
     <row r="12" spans="1:3" ht="16.5" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A12" s="13"/>
     </row>
-    <row r="14" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="2"/>
     </row>
-    <row r="16" spans="1:3" ht="15.75" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
         <v>0</v>
       </c>
@@ -3434,127 +3973,127 @@
         <v>2</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="62" t="s">
+    <row r="17" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="60" t="s">
         <v>66</v>
       </c>
-      <c r="B17" s="63" t="s">
+      <c r="B17" s="61" t="s">
         <v>67</v>
       </c>
-      <c r="C17" s="64"/>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A18" s="65" t="s">
+      <c r="C17" s="62"/>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" s="63" t="s">
         <v>68</v>
       </c>
-      <c r="B18" s="66" t="s">
+      <c r="B18" s="64" t="s">
         <v>69</v>
       </c>
-      <c r="C18" s="67"/>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A19" s="65" t="s">
+      <c r="C18" s="65"/>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" s="63" t="s">
         <v>70</v>
       </c>
-      <c r="B19" s="68">
+      <c r="B19" s="66">
         <v>31</v>
       </c>
-      <c r="C19" s="67" t="s">
+      <c r="C19" s="65" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A20" s="65" t="s">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" s="63" t="s">
         <v>72</v>
       </c>
-      <c r="B20" s="68">
+      <c r="B20" s="66">
         <v>47</v>
       </c>
-      <c r="C20" s="67" t="s">
+      <c r="C20" s="65" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A21" s="65" t="s">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" s="63" t="s">
         <v>74</v>
       </c>
-      <c r="B21" s="68">
+      <c r="B21" s="66">
         <v>1460</v>
       </c>
-      <c r="C21" s="67" t="s">
+      <c r="C21" s="65" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A22" s="65" t="s">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" s="63" t="s">
         <v>76</v>
       </c>
-      <c r="B22" s="68">
+      <c r="B22" s="66">
         <v>28.1</v>
       </c>
-      <c r="C22" s="67" t="s">
+      <c r="C22" s="65" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A23" s="65" t="s">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" s="63" t="s">
         <v>77</v>
       </c>
-      <c r="B23" s="68">
+      <c r="B23" s="66">
         <v>40.200000000000003</v>
       </c>
-      <c r="C23" s="67" t="s">
+      <c r="C23" s="65" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A24" s="65" t="s">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" s="63" t="s">
         <v>78</v>
       </c>
-      <c r="B24" s="69">
+      <c r="B24" s="67">
         <v>1.68E-6</v>
       </c>
-      <c r="C24" s="67" t="s">
+      <c r="C24" s="65" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A25" s="65" t="s">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" s="63" t="s">
         <v>80</v>
       </c>
-      <c r="B25" s="69" t="s">
-        <v>153</v>
-      </c>
-      <c r="C25" s="67" t="s">
+      <c r="B25" s="67" t="s">
+        <v>155</v>
+      </c>
+      <c r="C25" s="65" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A26" s="70" t="s">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" s="68" t="s">
         <v>82</v>
       </c>
-      <c r="B26" s="71">
+      <c r="B26" s="69">
         <v>1510</v>
       </c>
-      <c r="C26" s="67"/>
-    </row>
-    <row r="27" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="72" t="s">
+      <c r="C26" s="65"/>
+    </row>
+    <row r="27" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="70" t="s">
         <v>83</v>
       </c>
-      <c r="B27" s="73">
+      <c r="B27" s="71">
         <v>0.65</v>
       </c>
-      <c r="C27" s="74"/>
-    </row>
-    <row r="28" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.2"/>
-    <row r="30" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+      <c r="C27" s="72"/>
+    </row>
+    <row r="28" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="30" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="32" spans="1:3" ht="15.75" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="32" spans="1:3" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="3" t="s">
         <v>0</v>
       </c>
@@ -3565,179 +4104,186 @@
         <v>7</v>
       </c>
     </row>
-    <row r="33" spans="1:7" ht="15" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="62" t="s">
+    <row r="33" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="60" t="s">
         <v>85</v>
       </c>
-      <c r="B33" s="75">
+      <c r="B33" s="73">
         <v>0.1</v>
       </c>
-      <c r="C33" s="76" t="s">
+      <c r="C33" s="74" t="s">
         <v>145</v>
       </c>
-      <c r="G33" s="77"/>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A34" s="78" t="s">
+      <c r="G33" s="75"/>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34" s="76" t="s">
         <v>86</v>
       </c>
-      <c r="B34" s="79">
+      <c r="B34" s="77">
         <v>12</v>
       </c>
-      <c r="C34" s="80" t="s">
+      <c r="C34" s="78" t="s">
         <v>146</v>
       </c>
-      <c r="G34" s="77"/>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A35" s="78" t="s">
+      <c r="G34" s="75"/>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" s="76" t="s">
         <v>87</v>
       </c>
-      <c r="B35" s="81">
+      <c r="B35" s="79">
         <v>0.22600000000000001</v>
       </c>
-      <c r="C35" s="80" t="s">
+      <c r="C35" s="78" t="s">
         <v>147</v>
       </c>
-      <c r="F35" s="82"/>
-      <c r="G35" s="77"/>
+      <c r="F35" s="80"/>
+      <c r="G35" s="75"/>
     </row>
     <row r="36" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A36" s="78" t="s">
+      <c r="A36" s="76" t="s">
         <v>88</v>
       </c>
-      <c r="B36" s="83" t="str">
+      <c r="B36" s="81" t="str">
         <f>IF(B35&lt;=B10,"Yes","No")</f>
         <v>Yes</v>
       </c>
-      <c r="C36" s="80"/>
+      <c r="C36" s="78"/>
       <c r="E36" s="13"/>
       <c r="F36" s="13"/>
       <c r="G36" s="13"/>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A37" s="78" t="s">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A37" s="76" t="s">
         <v>89</v>
       </c>
-      <c r="B37" s="79">
+      <c r="B37" s="77">
         <v>0.20599999999999999</v>
       </c>
-      <c r="C37" s="80" t="s">
+      <c r="C37" s="78" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A38" s="85" t="s">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A38" s="83" t="s">
         <v>97</v>
       </c>
-      <c r="B38" s="84">
+      <c r="B38" s="82">
         <v>0.5</v>
       </c>
-      <c r="C38" s="80" t="s">
+      <c r="C38" s="78" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A39" s="85" t="s">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A39" s="83" t="s">
         <v>96</v>
       </c>
-      <c r="B39" s="79">
+      <c r="B39" s="77">
         <v>0.98199999999999998</v>
       </c>
-      <c r="C39" s="80" t="s">
+      <c r="C39" s="78" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A40" s="85" t="s">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A40" s="83" t="s">
         <v>98</v>
       </c>
-      <c r="B40" s="84">
+      <c r="B40" s="82">
         <v>5</v>
       </c>
-      <c r="C40" s="80"/>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A41" s="85" t="s">
+      <c r="C40" s="78"/>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A41" s="83" t="s">
         <v>99</v>
       </c>
-      <c r="B41" s="79">
+      <c r="B41" s="77">
         <v>8.2550000000000008</v>
       </c>
-      <c r="C41" s="80" t="s">
+      <c r="C41" s="78" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="42" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="87" t="s">
+    <row r="42" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="84" t="s">
         <v>90</v>
       </c>
-      <c r="B42" s="88">
+      <c r="B42" s="85">
         <v>0.33</v>
       </c>
-      <c r="C42" s="89" t="s">
+      <c r="C42" s="86" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="43" spans="1:7" ht="15" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="B43" s="77"/>
-    </row>
-    <row r="45" spans="1:7" ht="18" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="B43" s="75"/>
+    </row>
+    <row r="45" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="46" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="47" spans="1:7" ht="15.75" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="47" spans="1:7" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B47" s="3" t="s">
+      <c r="B47" s="95" t="s">
         <v>1</v>
       </c>
       <c r="C47" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="48" spans="1:7" ht="15" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="85" t="s">
+    <row r="48" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="89" t="s">
         <v>101</v>
       </c>
-      <c r="B48" s="79"/>
-      <c r="C48" s="80" t="s">
+      <c r="B48" s="88">
+        <v>39</v>
+      </c>
+      <c r="C48" s="92" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A49" s="78" t="s">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A49" s="90" t="s">
         <v>87</v>
       </c>
-      <c r="B49" s="93"/>
-      <c r="C49" s="67" t="s">
+      <c r="B49" s="96">
+        <v>0.248</v>
+      </c>
+      <c r="C49" s="93" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A50" s="85" t="s">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A50" s="89" t="s">
         <v>152</v>
       </c>
-      <c r="B50" s="93"/>
-      <c r="C50" s="67" t="s">
+      <c r="B50" s="96">
+        <v>7.5</v>
+      </c>
+      <c r="C50" s="93" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="51" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="86" t="s">
+    <row r="51" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A51" s="91" t="s">
         <v>102</v>
       </c>
-      <c r="B51" s="91"/>
-      <c r="C51" s="92" t="s">
+      <c r="B51" s="97">
+        <v>12</v>
+      </c>
+      <c r="C51" s="94" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="52" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.2"/>
+    <row r="52" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>